<commit_message>
fix(editorial): E9 Push 2 tail — §5.4 ge/gij imperative sweep (5 cells)
Cole-Machine bare-stem imperatives previously missed by e9 scanner
(regex only matched "Stop"). Broader sweep across all ge/gij speakers
caught 5 cells in BadCave + GoldenAss:

  J34 Geef → Geeft
  J63 Stop → Stopt
  J64 Probeer → Probeert (+ §7.3 machine → Machine)
  J81 Luister → Luistert
  J135 Ga → Gaat (gaan irregular)

Verified-clean cases where stem ends in -t (Wacht, Laat): no doubling.

Canon §19 E9 row updated. Canon §23 J63/J64 notes flipped to resolved.

Round-trip: 0 diffs / 5 cells.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excels/9_asses.masses_E9Proxy.xlsx
+++ b/excels/9_asses.masses_E9Proxy.xlsx
@@ -17888,7 +17888,7 @@
       </c>
       <c r="J34" s="44" t="inlineStr">
         <is>
-          <t>'k Start de initializer op. Geef mij een minuutje.</t>
+          <t>'k Start de initializer op. Geeft mij een minuutje.</t>
         </is>
       </c>
       <c r="K34" s="34" t="inlineStr">
@@ -19570,7 +19570,7 @@
       </c>
       <c r="J63" s="45" t="inlineStr">
         <is>
-          <t>Stevige. Stop.</t>
+          <t>Stevige. Stopt.</t>
         </is>
       </c>
       <c r="K63" s="34" t="inlineStr">
@@ -19628,7 +19628,7 @@
       </c>
       <c r="J64" s="45" t="inlineStr">
         <is>
-          <t>Probeer de machine niet kapot te maken.</t>
+          <t>Probeert de Machine niet kapot te maken.</t>
         </is>
       </c>
       <c r="K64" s="34" t="inlineStr">
@@ -20614,7 +20614,7 @@
       </c>
       <c r="J81" s="45" t="inlineStr">
         <is>
-          <t>Luister Stevige.</t>
+          <t>Luistert Stevige.</t>
         </is>
       </c>
       <c r="K81" s="34" t="inlineStr">
@@ -54044,7 +54044,7 @@
       </c>
       <c r="J135" s="45" t="inlineStr">
         <is>
-          <t>Ga dan.</t>
+          <t>Gaat dan.</t>
         </is>
       </c>
       <c r="K135" s="67" t="inlineStr">

</xml_diff>